<commit_message>
puzzles: refine bead loop color and sizing
</commit_message>
<xml_diff>
--- a/task-reviews/puzzles/task_puzzles_topology_bead_equivalence_count/task_puzzles_topology_bead_equivalence_count.xlsx
+++ b/task-reviews/puzzles/task_puzzles_topology_bead_equivalence_count/task_puzzles_topology_bead_equivalence_count.xlsx
@@ -4304,12 +4304,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -4432,12 +4432,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [314.0, 578.0, 486.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [314.0, 578.0, 486.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -4496,12 +4496,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 578.0, 486.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[714.0, 578.0, 886.0, 732.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 578.0, 486.0, 732.0]]</t>
+          <t>[[714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -4560,12 +4560,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[614.0, 578.0, 786.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[414.0, 578.0, 586.0, 732.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -4624,12 +4624,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4688,12 +4688,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]], "answer": 2}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -4816,12 +4816,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4880,12 +4880,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[614.0, 348.0, 786.0, 502.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4944,12 +4944,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -5008,12 +5008,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -5072,12 +5072,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -5136,12 +5136,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[414.0, 578.0, 586.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[814.0, 348.0, 986.0, 502.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[414.0, 578.0, 586.0, 732.0]]</t>
+          <t>[[814.0, 348.0, 986.0, 502.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -5200,12 +5200,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -5264,12 +5264,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[814.0, 348.0, 986.0, 502.0], [414.0, 578.0, 586.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[814.0, 348.0, 986.0, 502.0], [414.0, 578.0, 586.0, 732.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -5392,12 +5392,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5456,12 +5456,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5520,12 +5520,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 578.0, 386.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 578.0, 386.0, 732.0]]</t>
+          <t>[[614.0, 348.0, 786.0, 502.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5584,12 +5584,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]], "answer": 3}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5648,12 +5648,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5712,12 +5712,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 578.0, 886.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5776,12 +5776,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -5840,12 +5840,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -6001,12 +6001,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [314.0, 578.0, 486.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [314.0, 578.0, 486.0, 732.0]]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -6065,12 +6065,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6129,12 +6129,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 578.0, 386.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 578.0, 386.0, 732.0]]</t>
+          <t>[[614.0, 348.0, 786.0, 502.0]]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6193,12 +6193,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [414.0, 578.0, 586.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [414.0, 578.0, 586.0, 732.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [414.0, 578.0, 586.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6257,12 +6257,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -6321,12 +6321,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0]], "answer": 3}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6385,12 +6385,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -6449,12 +6449,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 578.0, 886.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -6513,12 +6513,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -6577,12 +6577,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -6641,12 +6641,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -6705,12 +6705,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0]], "answer": 1}</t>
+          <t>{"evidence": [[214.0, 578.0, 386.0, 732.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>[[614.0, 348.0, 786.0, 502.0]]</t>
+          <t>[[214.0, 578.0, 386.0, 732.0]]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -6769,12 +6769,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -6833,12 +6833,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 578.0, 486.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[714.0, 578.0, 886.0, 732.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 578.0, 486.0, 732.0]]</t>
+          <t>[[714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -6897,12 +6897,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>[[714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0]]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -6961,12 +6961,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [414.0, 578.0, 586.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -7025,12 +7025,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]], "answer": 2}</t>
+          <t>{"evidence": [[214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]]</t>
+          <t>[[214.0, 578.0, 386.0, 732.0], [614.0, 578.0, 786.0, 732.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -7089,12 +7089,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [414.0, 578.0, 586.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[814.0, 348.0, 986.0, 502.0], [214.0, 578.0, 386.0, 732.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -7153,12 +7153,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -7217,12 +7217,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -7281,12 +7281,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]], "answer": 2}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 578.0, 586.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -7409,12 +7409,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -7473,12 +7473,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -7537,12 +7537,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 5}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]], "answer": 5}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [314.0, 578.0, 486.0, 732.0], [514.0, 578.0, 686.0, 732.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -7762,12 +7762,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0]], "answer": 1}</t>
+          <t>{"evidence": [[214.0, 578.0, 386.0, 732.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>[[614.0, 348.0, 786.0, 502.0]]</t>
+          <t>[[214.0, 578.0, 386.0, 732.0]]</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7890,12 +7890,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[514.0, 578.0, 686.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[[514.0, 578.0, 686.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0]]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -8082,12 +8082,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>[[414.0, 348.0, 586.0, 502.0], [614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -8146,12 +8146,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [414.0, 578.0, 586.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [414.0, 578.0, 586.0, 732.0]]</t>
+          <t>[[614.0, 348.0, 786.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -8274,12 +8274,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [714.0, 578.0, 886.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>[[514.0, 348.0, 686.0, 502.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0]]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -8338,12 +8338,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [214.0, 578.0, 386.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [614.0, 348.0, 786.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [214.0, 578.0, 386.0, 732.0]]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -8466,12 +8466,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [814.0, 348.0, 986.0, 502.0], [614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 348.0, 386.0, 502.0], [414.0, 348.0, 586.0, 502.0], [214.0, 578.0, 386.0, 732.0], [414.0, 578.0, 586.0, 732.0]]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -8530,12 +8530,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -8722,12 +8722,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0]], "answer": 3}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 3}</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [514.0, 578.0, 686.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -8786,12 +8786,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[614.0, 578.0, 786.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[214.0, 578.0, 386.0, 732.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>[[614.0, 578.0, 786.0, 732.0]]</t>
+          <t>[[214.0, 578.0, 386.0, 732.0]]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -8914,12 +8914,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
+          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]], "answer": 4}</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]]</t>
+          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -8978,12 +8978,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 348.0, 486.0, 502.0], [514.0, 578.0, 686.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 348.0, 486.0, 502.0], [514.0, 578.0, 686.0, 732.0]]</t>
+          <t>[[714.0, 348.0, 886.0, 502.0], [714.0, 578.0, 886.0, 732.0]]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -9042,12 +9042,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[314.0, 578.0, 486.0, 732.0]], "answer": 1}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>[[314.0, 578.0, 486.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0]]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -9106,12 +9106,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0]], "answer": 2}</t>
+          <t>{"evidence": [[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0]], "answer": 2}</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>[[714.0, 348.0, 886.0, 502.0], [514.0, 578.0, 686.0, 732.0]]</t>
+          <t>[[514.0, 348.0, 686.0, 502.0], [314.0, 578.0, 486.0, 732.0]]</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -9170,12 +9170,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[614.0, 348.0, 786.0, 502.0]], "answer": 1}</t>
+          <t>{"evidence": [[214.0, 578.0, 386.0, 732.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>[[614.0, 348.0, 786.0, 502.0]]</t>
+          <t>[[214.0, 578.0, 386.0, 732.0]]</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -9234,12 +9234,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>{"evidence": [[814.0, 348.0, 986.0, 502.0]], "answer": 1}</t>
+          <t>{"evidence": [[414.0, 348.0, 586.0, 502.0]], "answer": 1}</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>[[814.0, 348.0, 986.0, 502.0]]</t>
+          <t>[[414.0, 348.0, 586.0, 502.0]]</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">

</xml_diff>